<commit_message>
Show split shares in the experimental results workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/model_development/results/Experimental_results.xlsx
+++ b/model_development/results/Experimental_results.xlsx
@@ -833,8 +833,10 @@
           <t>Training samples</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
-        <v>9077</v>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>9,077 (79.9%)</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -843,8 +845,10 @@
           <t>Validation samples</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
-        <v>1108</v>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>1,108 (9.8%)</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -853,8 +857,10 @@
           <t>Test samples</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n">
-        <v>1175</v>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>1,175 (10.3%)</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -1243,8 +1249,10 @@
           <t>Training samples</t>
         </is>
       </c>
-      <c r="B19" s="3" t="n">
-        <v>8611</v>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>8,611 (80.2%)</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -1253,8 +1261,10 @@
           <t>Validation samples</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n">
-        <v>1059</v>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>1,059 (9.9%)</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -1263,8 +1273,10 @@
           <t>Test samples</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n">
-        <v>1070</v>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>1,070 (10.0%)</t>
+        </is>
       </c>
     </row>
     <row r="22">

</xml_diff>